<commit_message>
add column to coupon_import.xlsx
</commit_message>
<xml_diff>
--- a/coupon_import.xlsx
+++ b/coupon_import.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matteo/code/projects/game_of_life/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27AFF7E-320F-E042-908B-175489F8CD91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="3540" yWindow="760" windowWidth="15960" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="64">
   <si>
     <t>Coupon ID</t>
   </si>
@@ -200,29 +209,21 @@
   </si>
   <si>
     <t>Iphone</t>
+  </si>
+  <si>
+    <t>new col</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="0" formatCode="General"/>
-    <numFmt numFmtId="59" formatCode="d/m/yy&quot; &quot;h:mm"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="d/m/yy&quot; &quot;h:mm"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="15"/>
       <color indexed="8"/>
       <name val="Calibri"/>
     </font>
@@ -356,59 +357,28 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs count="17">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="16">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="59" fontId="0" fillId="2" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -417,26 +387,85 @@
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffaaaaaa"/>
-      <rgbColor rgb="ff333333"/>
-      <rgbColor rgb="ffff0000"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFAAAAAA"/>
+      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office Theme">
       <a:dk1>
@@ -638,7 +667,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -657,7 +686,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -687,7 +716,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -713,7 +742,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -739,7 +768,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -765,7 +794,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -791,7 +820,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -817,7 +846,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -843,7 +872,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -869,7 +898,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -895,7 +924,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -908,9 +937,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -927,7 +962,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -946,7 +981,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -972,7 +1007,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -998,7 +1033,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1024,7 +1059,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1050,7 +1085,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1076,7 +1111,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1102,7 +1137,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1128,7 +1163,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1154,7 +1189,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1180,7 +1215,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1193,9 +1228,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -1209,7 +1250,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1228,7 +1269,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1258,7 +1299,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1284,7 +1325,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1310,7 +1351,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1336,7 +1377,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1362,7 +1403,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1388,7 +1429,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1414,7 +1455,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1440,7 +1481,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1466,7 +1507,7 @@
           <a:buFontTx/>
           <a:buNone/>
           <a:tabLst/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1479,191 +1520,201 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AV46"/>
-  <sheetFormatPr defaultColWidth="10.8333" defaultRowHeight="16" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AW46"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.8516" style="1" customWidth="1"/>
-    <col min="2" max="4" width="76.6719" style="1" customWidth="1"/>
-    <col min="5" max="6" width="10.8516" style="1" customWidth="1"/>
-    <col min="7" max="8" width="29.8516" style="1" customWidth="1"/>
-    <col min="9" max="10" width="64.6719" style="1" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" style="1" customWidth="1"/>
+    <col min="2" max="4" width="76.6640625" style="1" customWidth="1"/>
+    <col min="5" max="6" width="10.83203125" style="1" customWidth="1"/>
+    <col min="7" max="8" width="29.83203125" style="1" customWidth="1"/>
+    <col min="9" max="10" width="64.6640625" style="1" customWidth="1"/>
     <col min="11" max="11" width="26.5" style="1" customWidth="1"/>
-    <col min="12" max="12" width="55.8516" style="1" customWidth="1"/>
-    <col min="13" max="13" width="10.8516" style="1" customWidth="1"/>
-    <col min="14" max="14" width="20.1719" style="1" customWidth="1"/>
-    <col min="15" max="17" width="10.8516" style="1" customWidth="1"/>
-    <col min="18" max="18" width="17.1719" style="1" customWidth="1"/>
+    <col min="12" max="12" width="55.83203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="10.83203125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="20.1640625" style="1" customWidth="1"/>
+    <col min="15" max="17" width="10.83203125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="17.1640625" style="1" customWidth="1"/>
     <col min="19" max="19" width="20.5" style="1" customWidth="1"/>
-    <col min="20" max="35" width="10.8516" style="1" customWidth="1"/>
-    <col min="36" max="36" width="20.3516" style="1" customWidth="1"/>
+    <col min="20" max="35" width="10.83203125" style="1" customWidth="1"/>
+    <col min="36" max="36" width="20.33203125" style="1" customWidth="1"/>
     <col min="37" max="37" width="21.5" style="1" customWidth="1"/>
     <col min="38" max="38" width="19.5" style="1" customWidth="1"/>
-    <col min="39" max="39" width="14.8516" style="1" customWidth="1"/>
-    <col min="40" max="42" width="10.8516" style="1" customWidth="1"/>
-    <col min="43" max="43" width="32.3516" style="1" customWidth="1"/>
-    <col min="44" max="48" width="10.8516" style="1" customWidth="1"/>
-    <col min="49" max="16384" width="10.8516" style="1" customWidth="1"/>
+    <col min="39" max="39" width="14.83203125" style="1" customWidth="1"/>
+    <col min="40" max="42" width="10.83203125" style="1" customWidth="1"/>
+    <col min="43" max="43" width="32.33203125" style="1" customWidth="1"/>
+    <col min="44" max="49" width="10.83203125" style="1" customWidth="1"/>
+    <col min="50" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.25" customHeight="1">
-      <c r="A1" t="s" s="2">
+    <row r="1" spans="1:49" ht="15.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="3">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="3">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="3">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="4">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="3">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s" s="5">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s" s="5">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s" s="3">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s" s="3">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s" s="3">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s" s="3">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s" s="3">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s" s="3">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s" s="3">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s" s="3">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s" s="3">
+      <c r="Q1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s" s="3">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s" s="3">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s" s="3">
+      <c r="T1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s" s="3">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s" s="3">
+      <c r="V1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s" s="3">
+      <c r="W1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s" s="3">
+      <c r="X1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s" s="3">
+      <c r="Y1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s" s="3">
+      <c r="Z1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s" s="3">
+      <c r="AA1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" t="s" s="3">
+      <c r="AB1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" t="s" s="3">
+      <c r="AC1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" t="s" s="3">
+      <c r="AD1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" t="s" s="3">
+      <c r="AE1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" t="s" s="3">
+      <c r="AF1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" t="s" s="3">
+      <c r="AG1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" t="s" s="3">
+      <c r="AH1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" t="s" s="3">
+      <c r="AI1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" t="s" s="3">
+      <c r="AJ1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" t="s" s="3">
+      <c r="AK1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" t="s" s="3">
+      <c r="AL1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" t="s" s="3">
+      <c r="AM1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" t="s" s="3">
+      <c r="AN1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" t="s" s="3">
+      <c r="AO1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" t="s" s="3">
+      <c r="AP1" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" t="s" s="3">
+      <c r="AQ1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" t="s" s="3">
+      <c r="AR1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" t="s" s="3">
+      <c r="AS1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" t="s" s="3">
+      <c r="AT1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" t="s" s="6">
+      <c r="AU1" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" t="s" s="7">
+      <c r="AV1" s="7" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
+      <c r="AW1" s="16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8"/>
       <c r="B2" s="9">
         <v>1</v>
@@ -1671,46 +1722,46 @@
       <c r="C2" s="9">
         <v>1</v>
       </c>
-      <c r="D2" t="s" s="10">
+      <c r="D2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E2" t="s" s="11">
+      <c r="E2" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="F2" t="s" s="10">
+      <c r="F2" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="G2" t="s" s="10">
+      <c r="G2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="H2" t="s" s="10">
+      <c r="H2" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="I2" t="s" s="10">
+      <c r="I2" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="J2" t="s" s="10">
+      <c r="J2" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="K2" t="s" s="10">
+      <c r="K2" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="L2" t="s" s="10">
+      <c r="L2" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="M2" t="s" s="10">
+      <c r="M2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="N2" t="s" s="10">
+      <c r="N2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="O2" t="s" s="10">
+      <c r="O2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="P2" t="s" s="10">
+      <c r="P2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="Q2" t="s" s="10">
+      <c r="Q2" s="10" t="s">
         <v>48</v>
       </c>
       <c r="R2" s="12">
@@ -1719,93 +1770,96 @@
       <c r="S2" s="12">
         <v>43465.916666666664</v>
       </c>
-      <c r="T2" t="s" s="10">
+      <c r="T2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="U2" t="s" s="10">
+      <c r="U2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="V2" t="s" s="10">
+      <c r="V2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="W2" t="s" s="10">
+      <c r="W2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="X2" t="s" s="10">
+      <c r="X2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="Y2" t="s" s="10">
+      <c r="Y2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="Z2" t="s" s="10">
+      <c r="Z2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="AA2" t="s" s="10">
+      <c r="AA2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="AB2" t="s" s="10">
+      <c r="AB2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="AC2" t="s" s="10">
+      <c r="AC2" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="AD2" t="s" s="10">
+      <c r="AD2" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="AE2" t="s" s="10">
+      <c r="AE2" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="AF2" t="s" s="10">
+      <c r="AF2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="AG2" t="s" s="10">
+      <c r="AG2" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="AH2" t="s" s="10">
+      <c r="AH2" s="10" t="s">
         <v>55</v>
       </c>
       <c r="AI2" s="8"/>
-      <c r="AJ2" t="s" s="10">
+      <c r="AJ2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="AK2" t="s" s="10">
+      <c r="AK2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="AL2" t="s" s="10">
+      <c r="AL2" s="10" t="s">
         <v>48</v>
       </c>
       <c r="AM2" s="9">
         <v>2</v>
       </c>
-      <c r="AN2" t="s" s="10">
+      <c r="AN2" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="AO2" t="s" s="10">
+      <c r="AO2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="AP2" t="s" s="10">
+      <c r="AP2" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="AQ2" t="s" s="10">
+      <c r="AQ2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="AR2" t="s" s="10">
+      <c r="AR2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="AS2" t="s" s="10">
+      <c r="AS2" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="AT2" t="s" s="10">
+      <c r="AT2" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="AU2" t="s" s="10">
+      <c r="AU2" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="AV2" t="s" s="13">
+      <c r="AV2" s="13" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
+      <c r="AW2" s="13" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="14"/>
       <c r="B3" s="14"/>
       <c r="C3" s="14"/>
@@ -1855,7 +1909,7 @@
       <c r="AU3" s="14"/>
       <c r="AV3" s="15"/>
     </row>
-    <row r="4" ht="16" customHeight="1">
+    <row r="4" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="14"/>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
@@ -1905,7 +1959,7 @@
       <c r="AU4" s="14"/>
       <c r="AV4" s="15"/>
     </row>
-    <row r="5" ht="16" customHeight="1">
+    <row r="5" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="14"/>
       <c r="B5" s="14"/>
       <c r="C5" s="14"/>
@@ -1955,7 +2009,7 @@
       <c r="AU5" s="14"/>
       <c r="AV5" s="15"/>
     </row>
-    <row r="6" ht="16" customHeight="1">
+    <row r="6" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="14"/>
       <c r="B6" s="14"/>
       <c r="C6" s="14"/>
@@ -2005,7 +2059,7 @@
       <c r="AU6" s="14"/>
       <c r="AV6" s="15"/>
     </row>
-    <row r="7" ht="16" customHeight="1">
+    <row r="7" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="14"/>
       <c r="B7" s="14"/>
       <c r="C7" s="14"/>
@@ -2055,7 +2109,7 @@
       <c r="AU7" s="14"/>
       <c r="AV7" s="15"/>
     </row>
-    <row r="8" ht="16" customHeight="1">
+    <row r="8" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="14"/>
       <c r="B8" s="14"/>
       <c r="C8" s="14"/>
@@ -2105,7 +2159,7 @@
       <c r="AU8" s="14"/>
       <c r="AV8" s="15"/>
     </row>
-    <row r="9" ht="16" customHeight="1">
+    <row r="9" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="14"/>
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
@@ -2155,7 +2209,7 @@
       <c r="AU9" s="14"/>
       <c r="AV9" s="15"/>
     </row>
-    <row r="10" ht="16" customHeight="1">
+    <row r="10" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="14"/>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
@@ -2205,7 +2259,7 @@
       <c r="AU10" s="14"/>
       <c r="AV10" s="15"/>
     </row>
-    <row r="11" ht="16" customHeight="1">
+    <row r="11" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="14"/>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
@@ -2255,7 +2309,7 @@
       <c r="AU11" s="14"/>
       <c r="AV11" s="15"/>
     </row>
-    <row r="12" ht="16" customHeight="1">
+    <row r="12" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="14"/>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
@@ -2305,7 +2359,7 @@
       <c r="AU12" s="14"/>
       <c r="AV12" s="15"/>
     </row>
-    <row r="13" ht="16" customHeight="1">
+    <row r="13" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="14"/>
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
@@ -2355,7 +2409,7 @@
       <c r="AU13" s="14"/>
       <c r="AV13" s="15"/>
     </row>
-    <row r="14" ht="16" customHeight="1">
+    <row r="14" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
@@ -2405,7 +2459,7 @@
       <c r="AU14" s="14"/>
       <c r="AV14" s="15"/>
     </row>
-    <row r="15" ht="16" customHeight="1">
+    <row r="15" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="14"/>
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
@@ -2455,7 +2509,7 @@
       <c r="AU15" s="14"/>
       <c r="AV15" s="15"/>
     </row>
-    <row r="16" ht="16" customHeight="1">
+    <row r="16" spans="1:49" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="14"/>
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
@@ -2505,7 +2559,7 @@
       <c r="AU16" s="14"/>
       <c r="AV16" s="15"/>
     </row>
-    <row r="17" ht="16" customHeight="1">
+    <row r="17" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="14"/>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
@@ -2555,7 +2609,7 @@
       <c r="AU17" s="14"/>
       <c r="AV17" s="15"/>
     </row>
-    <row r="18" ht="16" customHeight="1">
+    <row r="18" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="14"/>
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
@@ -2605,7 +2659,7 @@
       <c r="AU18" s="14"/>
       <c r="AV18" s="15"/>
     </row>
-    <row r="19" ht="16" customHeight="1">
+    <row r="19" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
@@ -2655,7 +2709,7 @@
       <c r="AU19" s="14"/>
       <c r="AV19" s="15"/>
     </row>
-    <row r="20" ht="16" customHeight="1">
+    <row r="20" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="14"/>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
@@ -2705,7 +2759,7 @@
       <c r="AU20" s="14"/>
       <c r="AV20" s="15"/>
     </row>
-    <row r="21" ht="16" customHeight="1">
+    <row r="21" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="14"/>
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
@@ -2755,7 +2809,7 @@
       <c r="AU21" s="14"/>
       <c r="AV21" s="15"/>
     </row>
-    <row r="22" ht="16" customHeight="1">
+    <row r="22" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="14"/>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
@@ -2805,7 +2859,7 @@
       <c r="AU22" s="14"/>
       <c r="AV22" s="15"/>
     </row>
-    <row r="23" ht="16" customHeight="1">
+    <row r="23" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="14"/>
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
@@ -2855,7 +2909,7 @@
       <c r="AU23" s="14"/>
       <c r="AV23" s="15"/>
     </row>
-    <row r="24" ht="16" customHeight="1">
+    <row r="24" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="14"/>
       <c r="B24" s="14"/>
       <c r="C24" s="14"/>
@@ -2905,7 +2959,7 @@
       <c r="AU24" s="14"/>
       <c r="AV24" s="15"/>
     </row>
-    <row r="25" ht="16" customHeight="1">
+    <row r="25" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="14"/>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
@@ -2955,7 +3009,7 @@
       <c r="AU25" s="14"/>
       <c r="AV25" s="15"/>
     </row>
-    <row r="26" ht="16" customHeight="1">
+    <row r="26" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="14"/>
       <c r="B26" s="14"/>
       <c r="C26" s="14"/>
@@ -3005,7 +3059,7 @@
       <c r="AU26" s="14"/>
       <c r="AV26" s="15"/>
     </row>
-    <row r="27" ht="16" customHeight="1">
+    <row r="27" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="14"/>
       <c r="B27" s="14"/>
       <c r="C27" s="14"/>
@@ -3055,7 +3109,7 @@
       <c r="AU27" s="14"/>
       <c r="AV27" s="15"/>
     </row>
-    <row r="28" ht="16" customHeight="1">
+    <row r="28" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="14"/>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>
@@ -3105,7 +3159,7 @@
       <c r="AU28" s="14"/>
       <c r="AV28" s="15"/>
     </row>
-    <row r="29" ht="16" customHeight="1">
+    <row r="29" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="14"/>
       <c r="B29" s="14"/>
       <c r="C29" s="14"/>
@@ -3155,7 +3209,7 @@
       <c r="AU29" s="14"/>
       <c r="AV29" s="15"/>
     </row>
-    <row r="30" ht="16" customHeight="1">
+    <row r="30" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="14"/>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>
@@ -3205,7 +3259,7 @@
       <c r="AU30" s="14"/>
       <c r="AV30" s="15"/>
     </row>
-    <row r="31" ht="16" customHeight="1">
+    <row r="31" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="14"/>
       <c r="B31" s="14"/>
       <c r="C31" s="14"/>
@@ -3255,7 +3309,7 @@
       <c r="AU31" s="14"/>
       <c r="AV31" s="15"/>
     </row>
-    <row r="32" ht="16" customHeight="1">
+    <row r="32" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -3305,7 +3359,7 @@
       <c r="AU32" s="14"/>
       <c r="AV32" s="15"/>
     </row>
-    <row r="33" ht="16" customHeight="1">
+    <row r="33" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="14"/>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -3355,7 +3409,7 @@
       <c r="AU33" s="14"/>
       <c r="AV33" s="15"/>
     </row>
-    <row r="34" ht="16" customHeight="1">
+    <row r="34" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="14"/>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
@@ -3405,7 +3459,7 @@
       <c r="AU34" s="14"/>
       <c r="AV34" s="15"/>
     </row>
-    <row r="35" ht="16" customHeight="1">
+    <row r="35" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="14"/>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
@@ -3455,7 +3509,7 @@
       <c r="AU35" s="14"/>
       <c r="AV35" s="15"/>
     </row>
-    <row r="36" ht="16" customHeight="1">
+    <row r="36" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="14"/>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
@@ -3505,7 +3559,7 @@
       <c r="AU36" s="14"/>
       <c r="AV36" s="15"/>
     </row>
-    <row r="37" ht="16" customHeight="1">
+    <row r="37" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="14"/>
       <c r="B37" s="14"/>
       <c r="C37" s="14"/>
@@ -3555,7 +3609,7 @@
       <c r="AU37" s="14"/>
       <c r="AV37" s="15"/>
     </row>
-    <row r="38" ht="16" customHeight="1">
+    <row r="38" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="14"/>
       <c r="B38" s="14"/>
       <c r="C38" s="14"/>
@@ -3605,7 +3659,7 @@
       <c r="AU38" s="14"/>
       <c r="AV38" s="15"/>
     </row>
-    <row r="39" ht="16" customHeight="1">
+    <row r="39" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="14"/>
       <c r="B39" s="14"/>
       <c r="C39" s="14"/>
@@ -3655,7 +3709,7 @@
       <c r="AU39" s="14"/>
       <c r="AV39" s="15"/>
     </row>
-    <row r="40" ht="16" customHeight="1">
+    <row r="40" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="14"/>
       <c r="B40" s="14"/>
       <c r="C40" s="14"/>
@@ -3705,7 +3759,7 @@
       <c r="AU40" s="14"/>
       <c r="AV40" s="15"/>
     </row>
-    <row r="41" ht="16" customHeight="1">
+    <row r="41" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="14"/>
       <c r="B41" s="14"/>
       <c r="C41" s="14"/>
@@ -3755,7 +3809,7 @@
       <c r="AU41" s="14"/>
       <c r="AV41" s="15"/>
     </row>
-    <row r="42" ht="16" customHeight="1">
+    <row r="42" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="14"/>
       <c r="B42" s="14"/>
       <c r="C42" s="14"/>
@@ -3805,7 +3859,7 @@
       <c r="AU42" s="14"/>
       <c r="AV42" s="15"/>
     </row>
-    <row r="43" ht="16" customHeight="1">
+    <row r="43" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="14"/>
       <c r="B43" s="14"/>
       <c r="C43" s="14"/>
@@ -3855,7 +3909,7 @@
       <c r="AU43" s="14"/>
       <c r="AV43" s="15"/>
     </row>
-    <row r="44" ht="16" customHeight="1">
+    <row r="44" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="14"/>
       <c r="B44" s="14"/>
       <c r="C44" s="14"/>
@@ -3905,7 +3959,7 @@
       <c r="AU44" s="14"/>
       <c r="AV44" s="15"/>
     </row>
-    <row r="45" ht="16" customHeight="1">
+    <row r="45" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="14"/>
       <c r="B45" s="14"/>
       <c r="C45" s="14"/>
@@ -3955,7 +4009,7 @@
       <c r="AU45" s="14"/>
       <c r="AV45" s="15"/>
     </row>
-    <row r="46" ht="16" customHeight="1">
+    <row r="46" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="14"/>
       <c r="B46" s="14"/>
       <c r="C46" s="14"/>
@@ -4007,7 +4061,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>